<commit_message>
vault: daily sync 2026-04-28 — new notes, agent configs, weekly summaries, financial files
</commit_message>
<xml_diff>
--- a/95 Файлы/Допуск. Айсберг/Допуск. Айсберг. Лифты.xlsx
+++ b/95 Файлы/Допуск. Айсберг/Допуск. Айсберг. Лифты.xlsx
@@ -757,7 +757,7 @@
       </c>
       <c r="K2" s="15"/>
       <c r="L2" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M2" s="21"/>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="K3" s="22"/>
       <c r="L3" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M3" s="22"/>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="K4" s="22"/>
       <c r="L4" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M4" s="22"/>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="K5" s="8"/>
       <c r="L5" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M5" s="8"/>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="K6" s="8"/>
       <c r="L6" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M6" s="8"/>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="K7" s="15"/>
       <c r="L7" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M7" s="21"/>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="K8" s="22"/>
       <c r="L8" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M8" s="22"/>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="K9" s="22"/>
       <c r="L9" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M9" s="22"/>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="K10" s="15"/>
       <c r="L10" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M10" s="21"/>
     </row>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="K11" s="15"/>
       <c r="L11" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M11" s="21"/>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="K12" s="22"/>
       <c r="L12" s="10">
-        <v>46142</v>
+        <v>46173</v>
       </c>
       <c r="M12" s="22"/>
     </row>

</xml_diff>